<commit_message>
Updating with random module to return random status
</commit_message>
<xml_diff>
--- a/Project_Test_Cases.xlsx
+++ b/Project_Test_Cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sg97976\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sg97976\Desktop\Mega_Project\Python_Megha_Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFDDE419-3A53-4578-8882-73D4D140F0D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EB921DD-719C-4957-A197-16062FC87283}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,10 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>Test_ID</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
   <si>
     <t>Input</t>
   </si>
@@ -36,22 +33,31 @@
     <t>Expected</t>
   </si>
   <si>
-    <t>TC01</t>
-  </si>
-  <si>
-    <t>LOCK</t>
-  </si>
-  <si>
-    <t>LOCKED</t>
-  </si>
-  <si>
-    <t>TC02</t>
-  </si>
-  <si>
-    <t>UNLOCK</t>
-  </si>
-  <si>
-    <t>UNLOCKED</t>
+    <t>TC_ID</t>
+  </si>
+  <si>
+    <t>TC_01</t>
+  </si>
+  <si>
+    <t>lock</t>
+  </si>
+  <si>
+    <t>Door Locked</t>
+  </si>
+  <si>
+    <t>TC_02</t>
+  </si>
+  <si>
+    <t>unlock</t>
+  </si>
+  <si>
+    <t>Door Unlocked</t>
+  </si>
+  <si>
+    <t>TC_03</t>
+  </si>
+  <si>
+    <t>TC_04</t>
   </si>
 </sst>
 </file>
@@ -383,7 +389,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.140625" customWidth="1"/>
@@ -392,13 +398,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -412,7 +418,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -420,6 +426,28 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>